<commit_message>
Update cellphone app data and add Galileos Secret
</commit_message>
<xml_diff>
--- a/data/image_data.xlsx
+++ b/data/image_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\dov-art-app\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Programming\MyCellphoeApp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F44872E7-23CA-40C9-B16B-5660266C102F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4198F74D-49A4-4E58-9210-F22BEB21B014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2460" windowWidth="17970" windowHeight="13740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="794">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="800">
   <si>
     <t>Number</t>
   </si>
@@ -2413,6 +2413,24 @@
   </si>
   <si>
     <t>How many selves do we imprison before we recognize the cage is inward?</t>
+  </si>
+  <si>
+    <t>The Frame Between Us</t>
+  </si>
+  <si>
+    <t>Galileos Secret</t>
+  </si>
+  <si>
+    <t>An elderly bald man stands on a balcony or rooftop terrace overlooking a Venetian canal at night, holding a modern digital camera with a telephoto lens. Beside him, an older bearded man in historical clothing looks through a long telescope, seemingly intent on some distant target. In the camera screen held by the modern visitor, however, the true object of attention is revealed: a blond woman, warmly lit and apparently bathing or undressing, caught from afar through the lens. Below and beyond them stretches a richly atmospheric Venetian cityscape of domes, towers, palaces, canals, and moored gondolas, illuminated by amber lights that reflect in the water. Above, a brilliant starry sky and a glowing comet heighten the mock-dramatic grandeur of the scene. On the stone table in the foreground lies an open old book inscribed Il Saggiatore 1623, along with diagrams and papers associated with learning and observation. The image combines historical costume, modern technology, romantic night scenery, and visual revelation into a theatrical and humorous tableau.</t>
+  </si>
+  <si>
+    <t>he image is a witty parody of observation, knowledge, and male curiosity. By presenting Galileo not as a heroic seeker of cosmic truth but as someone covertly using his telescope to watch a beautiful bathing woman, the work punctures the grandeur of science with humor and human weakness. The visitor from the future, instead of documenting the stars or Galileo’s discoveries, turns his camera toward Galileo’s hidden intention, exposing the absurdity of the scene. This creates a layered comedy of looking: the woman is watched by Galileo, Galileo is watched by the photographer, and the viewer watches them all. The telescope and camera become parallel instruments not of pure truth, but of desire, intrusion, and visual appropriation. Beneath the humor lies a sly comment on the continuity of human nature across centuries: technology changes, but curiosity, temptation, and the impulse to look remain the same. The image therefore works as both historical fantasy and visual joke, replacing reverence with irreverence and turning the mythology of genius into an affectionate, mischievous human comedy.</t>
+  </si>
+  <si>
+    <t>The Frame Between Us is set in a dim, textured interior space, where two versions of the same elderly man face one another across a quiet, symbolic divide. On the left, the man stands under an open black umbrella, gazing toward a large wooden frame mounted on the wall. Within the frame appears another version of himself, wearing a hat and standing calmly against a bright sky filled with soft clouds. A simple wooden ladder leans up toward the frame, suggesting a possible path between the two spaces. Above the man with the umbrella floats a solitary cloud inside the room, reinforcing the surreal atmosphere. The composition is sparse and carefully balanced, emphasizing the tension between the grounded interior and the luminous world visible through the frame.</t>
+  </si>
+  <si>
+    <t>The image explores the boundary between inner and outer worlds, reality and possibility, or present self and imagined self. The wooden frame functions as a portal rather than a mere picture frame, containing a version of the protagonist who appears serene and complete, bathed in open sky. The man inside the room, protected by an umbrella despite the absence of rain, embodies hesitation, caution, or emotional sheltering. The ladder introduces the idea of transition—an invitation to cross from introspection into openness—but its unused state suggests uncertainty or fear of change. The cloud hovering indoors further blurs the boundary between mental and physical spaces, implying that the weather of the mind has entered the room. Together, these elements create a meditation on self-confrontation: the moment when one stands before an image of who one might become and wonders whether the distance between the two selves can truly be climbed.</t>
   </si>
 </sst>
 </file>
@@ -2423,13 +2441,19 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2452,7 +2476,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2474,6 +2498,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2777,17 +2804,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G198"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="1" max="1" width="6" style="2" customWidth="1"/>
     <col min="2" max="2" width="34.25" customWidth="1"/>
     <col min="3" max="5" width="70" customWidth="1"/>
     <col min="6" max="6" width="14" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -2807,7 +2834,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="114" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
@@ -2827,7 +2854,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="327.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="A3" s="2">
         <f t="shared" ref="A3:A34" si="0">1+A2</f>
         <v>2</v>
       </c>
@@ -6935,8 +6962,36 @@
         <v>46087</v>
       </c>
     </row>
+    <row r="199" spans="1:7" ht="185.25" x14ac:dyDescent="0.2">
+      <c r="A199" s="2">
+        <v>198</v>
+      </c>
+      <c r="B199" t="s">
+        <v>794</v>
+      </c>
+      <c r="C199" s="1" t="s">
+        <v>798</v>
+      </c>
+      <c r="D199" s="1" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" ht="199.5" x14ac:dyDescent="0.2">
+      <c r="A200" s="2">
+        <v>199</v>
+      </c>
+      <c r="B200" t="s">
+        <v>795</v>
+      </c>
+      <c r="C200" s="8" t="s">
+        <v>796</v>
+      </c>
+      <c r="D200" s="8" t="s">
+        <v>797</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Against the Current image
</commit_message>
<xml_diff>
--- a/data/image_data.xlsx
+++ b/data/image_data.xlsx
@@ -1,36 +1,242 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Programming\dov-art-app\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9450448-D450-4909-90DB-1DE05276A74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>גליונות עבודה</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>גיליון1</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <cp:lastModifiedBy>Dov Fuchs</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2025-08-24T06:55:26Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-05-22T16:55:14Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\calcChain.xml><?xml version="1.0" encoding="utf-8"?>
+<calcChain xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <c r="A3" i="1" l="1"/>
+  <c r="A4" i="1" s="1"/>
+  <c r="A5" i="1" s="1"/>
+  <c r="A6" i="1" s="1"/>
+  <c r="A7" i="1" s="1"/>
+  <c r="A8" i="1" s="1"/>
+  <c r="A9" i="1" s="1"/>
+  <c r="A10" i="1" s="1"/>
+  <c r="A11" i="1" s="1"/>
+  <c r="A12" i="1" s="1"/>
+  <c r="A13" i="1" s="1"/>
+  <c r="A14" i="1" s="1"/>
+  <c r="A15" i="1" s="1"/>
+  <c r="A16" i="1" s="1"/>
+  <c r="A17" i="1" s="1"/>
+  <c r="A18" i="1" s="1"/>
+  <c r="A19" i="1" s="1"/>
+  <c r="A20" i="1" s="1"/>
+  <c r="A21" i="1" s="1"/>
+  <c r="A22" i="1" s="1"/>
+  <c r="A23" i="1" s="1"/>
+  <c r="A24" i="1" s="1"/>
+  <c r="A25" i="1" s="1"/>
+  <c r="A26" i="1" s="1"/>
+  <c r="A27" i="1" s="1"/>
+  <c r="A28" i="1" s="1"/>
+  <c r="A29" i="1" s="1"/>
+  <c r="A30" i="1" s="1"/>
+  <c r="A31" i="1" s="1"/>
+  <c r="A32" i="1" s="1"/>
+  <c r="A33" i="1" s="1"/>
+  <c r="A34" i="1" s="1"/>
+  <c r="A35" i="1" s="1"/>
+  <c r="A36" i="1" s="1"/>
+  <c r="A37" i="1" s="1"/>
+  <c r="A38" i="1" s="1"/>
+  <c r="A39" i="1" s="1"/>
+  <c r="A40" i="1" s="1"/>
+  <c r="A41" i="1" s="1"/>
+  <c r="A42" i="1" s="1"/>
+  <c r="A43" i="1" s="1"/>
+  <c r="A44" i="1" s="1"/>
+  <c r="A45" i="1" s="1"/>
+  <c r="A46" i="1" s="1"/>
+  <c r="A47" i="1" s="1"/>
+  <c r="A48" i="1" s="1"/>
+  <c r="A49" i="1" s="1"/>
+  <c r="A50" i="1" s="1"/>
+  <c r="A51" i="1" s="1"/>
+  <c r="A52" i="1" s="1"/>
+  <c r="A53" i="1" s="1"/>
+  <c r="A54" i="1" s="1"/>
+  <c r="A55" i="1" s="1"/>
+  <c r="A56" i="1" s="1"/>
+  <c r="A57" i="1" s="1"/>
+  <c r="A58" i="1" s="1"/>
+  <c r="A59" i="1" s="1"/>
+  <c r="A60" i="1" s="1"/>
+  <c r="A61" i="1" s="1"/>
+  <c r="A62" i="1" s="1"/>
+  <c r="A63" i="1" s="1"/>
+  <c r="A64" i="1" s="1"/>
+  <c r="A65" i="1" s="1"/>
+  <c r="A66" i="1" s="1"/>
+  <c r="A67" i="1" s="1"/>
+  <c r="A68" i="1" s="1"/>
+  <c r="A69" i="1" s="1"/>
+  <c r="A70" i="1" s="1"/>
+  <c r="A71" i="1" s="1"/>
+  <c r="A72" i="1" s="1"/>
+  <c r="A73" i="1" s="1"/>
+  <c r="A74" i="1" s="1"/>
+  <c r="A75" i="1" s="1"/>
+  <c r="A76" i="1" s="1"/>
+  <c r="A77" i="1" s="1"/>
+  <c r="A78" i="1" s="1"/>
+  <c r="A79" i="1" s="1"/>
+  <c r="A80" i="1" s="1"/>
+  <c r="A81" i="1" s="1"/>
+  <c r="A82" i="1" s="1"/>
+  <c r="A83" i="1" s="1"/>
+  <c r="A84" i="1" s="1"/>
+  <c r="A85" i="1" s="1"/>
+  <c r="A86" i="1" s="1"/>
+  <c r="A87" i="1" s="1"/>
+  <c r="A88" i="1" s="1"/>
+  <c r="A89" i="1" s="1"/>
+  <c r="A90" i="1" s="1"/>
+  <c r="A91" i="1" s="1"/>
+  <c r="A92" i="1" s="1"/>
+  <c r="A93" i="1" s="1"/>
+  <c r="A94" i="1" s="1"/>
+  <c r="A95" i="1" s="1"/>
+  <c r="A96" i="1" s="1"/>
+  <c r="A97" i="1" s="1"/>
+  <c r="A98" i="1" s="1"/>
+  <c r="A99" i="1" s="1"/>
+  <c r="A100" i="1" s="1"/>
+  <c r="A101" i="1" s="1"/>
+  <c r="A102" i="1" s="1"/>
+  <c r="A103" i="1" s="1"/>
+  <c r="A104" i="1" s="1"/>
+  <c r="A105" i="1" s="1"/>
+  <c r="A106" i="1" s="1"/>
+  <c r="A107" i="1" s="1"/>
+  <c r="A108" i="1" s="1"/>
+  <c r="A109" i="1" s="1"/>
+  <c r="A110" i="1" s="1"/>
+  <c r="A111" i="1" s="1"/>
+  <c r="A112" i="1" s="1"/>
+  <c r="A113" i="1" s="1"/>
+  <c r="A114" i="1" s="1"/>
+  <c r="A115" i="1" s="1"/>
+  <c r="A116" i="1" s="1"/>
+  <c r="A117" i="1" s="1"/>
+  <c r="A118" i="1" s="1"/>
+  <c r="A119" i="1" s="1"/>
+  <c r="A120" i="1" s="1"/>
+  <c r="A121" i="1" s="1"/>
+  <c r="A122" i="1" s="1"/>
+  <c r="A123" i="1" s="1"/>
+  <c r="A124" i="1" s="1"/>
+  <c r="A125" i="1" s="1"/>
+  <c r="A126" i="1" s="1"/>
+  <c r="A127" i="1" s="1"/>
+  <c r="A128" i="1" s="1"/>
+  <c r="A129" i="1" s="1"/>
+  <c r="A130" i="1" s="1"/>
+  <c r="A131" i="1" s="1"/>
+  <c r="A132" i="1" s="1"/>
+  <c r="A133" i="1" s="1"/>
+  <c r="A134" i="1" s="1"/>
+  <c r="A135" i="1" s="1"/>
+  <c r="A136" i="1" s="1"/>
+  <c r="A137" i="1" s="1"/>
+  <c r="A138" i="1" s="1"/>
+  <c r="A139" i="1" s="1"/>
+  <c r="A140" i="1" s="1"/>
+  <c r="A141" i="1" s="1"/>
+  <c r="A142" i="1" s="1"/>
+  <c r="A143" i="1" s="1"/>
+  <c r="A144" i="1" s="1"/>
+  <c r="A145" i="1" s="1"/>
+  <c r="A146" i="1" s="1"/>
+  <c r="A147" i="1" s="1"/>
+  <c r="A148" i="1" s="1"/>
+  <c r="A149" i="1" s="1"/>
+  <c r="A150" i="1" s="1"/>
+  <c r="A151" i="1" s="1"/>
+  <c r="A152" i="1" s="1"/>
+  <c r="A153" i="1" s="1"/>
+  <c r="A154" i="1" s="1"/>
+  <c r="A155" i="1" s="1"/>
+  <c r="A156" i="1" s="1"/>
+  <c r="A157" i="1" s="1"/>
+  <c r="A158" i="1" s="1"/>
+  <c r="A159" i="1" s="1"/>
+  <c r="A160" i="1" s="1"/>
+  <c r="A161" i="1" s="1"/>
+  <c r="A162" i="1" s="1"/>
+  <c r="A163" i="1" s="1"/>
+  <c r="A164" i="1" s="1"/>
+  <c r="A165" i="1" s="1"/>
+  <c r="A166" i="1" s="1"/>
+  <c r="A167" i="1" s="1"/>
+  <c r="A168" i="1" s="1"/>
+  <c r="A169" i="1" s="1"/>
+  <c r="A170" i="1" s="1"/>
+  <c r="A171" i="1" s="1"/>
+  <c r="A172" i="1" s="1"/>
+  <c r="A173" i="1" s="1"/>
+  <c r="A174" i="1" s="1"/>
+  <c r="A175" i="1" s="1"/>
+  <c r="A176" i="1" s="1"/>
+  <c r="A177" i="1" s="1"/>
+  <c r="A178" i="1" s="1"/>
+  <c r="A179" i="1" s="1"/>
+  <c r="A180" i="1" s="1"/>
+  <c r="A181" i="1" s="1"/>
+  <c r="A182" i="1" s="1"/>
+  <c r="A183" i="1" s="1"/>
+  <c r="A184" i="1" s="1"/>
+  <c r="A185" i="1" s="1"/>
+  <c r="A186" i="1" s="1"/>
+  <c r="A187" i="1" s="1"/>
+  <c r="A188" i="1" s="1"/>
+  <c r="A189" i="1" s="1"/>
+  <c r="A190" i="1" s="1"/>
+  <c r="A191" i="1" s="1"/>
+  <c r="A192" i="1" s="1"/>
+  <c r="A193" i="1" s="1"/>
+  <c r="A194" i="1" s="1"/>
+  <c r="A195" i="1" s="1"/>
+  <c r="A196" i="1" s="1"/>
+  <c r="A197" i="1" s="1"/>
+  <c r="A198" i="1" s="1"/>
+</calcChain>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="860">
   <si>
     <t>Number</t>
@@ -2661,7 +2867,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
@@ -2755,7 +2961,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -3038,7 +3244,38 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Programming\MyCellphoeApp\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77390DFE-F443-404A-BA9D-A23DC4070CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G215"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -7532,7 +7769,7 @@
         <v>859</v>
       </c>
       <c r="F215" s="5">
-        <v>374881</v>
+        <v>46163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Fifth Apple and sort by full date
</commit_message>
<xml_diff>
--- a/data/image_data.xlsx
+++ b/data/image_data.xlsx
@@ -1,243 +1,37 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>Microsoft Excel</Application>
-  <DocSecurity>0</DocSecurity>
-  <ScaleCrop>false</ScaleCrop>
-  <HeadingPairs>
-    <vt:vector size="2" baseType="variant">
-      <vt:variant>
-        <vt:lpstr>גליונות עבודה</vt:lpstr>
-      </vt:variant>
-      <vt:variant>
-        <vt:i4>1</vt:i4>
-      </vt:variant>
-    </vt:vector>
-  </HeadingPairs>
-  <TitlesOfParts>
-    <vt:vector size="1" baseType="lpstr">
-      <vt:lpstr>גיליון1</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-  <LinksUpToDate>false</LinksUpToDate>
-  <SharedDoc>false</SharedDoc>
-  <HyperlinksChanged>false</HyperlinksChanged>
-  <AppVersion>16.0300</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Programming\MyCellphoeApp\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB73146-E38F-40B7-86E7-B3B4E16CE8DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <dc:creator>openpyxl</dc:creator>
-  <cp:lastModifiedBy>Dov Fuchs</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2025-08-24T06:55:26Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-05-22T16:55:14Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=xl\calcChain.xml><?xml version="1.0" encoding="utf-8"?>
-<calcChain xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <c r="A3" i="1" l="1"/>
-  <c r="A4" i="1" s="1"/>
-  <c r="A5" i="1" s="1"/>
-  <c r="A6" i="1" s="1"/>
-  <c r="A7" i="1" s="1"/>
-  <c r="A8" i="1" s="1"/>
-  <c r="A9" i="1" s="1"/>
-  <c r="A10" i="1" s="1"/>
-  <c r="A11" i="1" s="1"/>
-  <c r="A12" i="1" s="1"/>
-  <c r="A13" i="1" s="1"/>
-  <c r="A14" i="1" s="1"/>
-  <c r="A15" i="1" s="1"/>
-  <c r="A16" i="1" s="1"/>
-  <c r="A17" i="1" s="1"/>
-  <c r="A18" i="1" s="1"/>
-  <c r="A19" i="1" s="1"/>
-  <c r="A20" i="1" s="1"/>
-  <c r="A21" i="1" s="1"/>
-  <c r="A22" i="1" s="1"/>
-  <c r="A23" i="1" s="1"/>
-  <c r="A24" i="1" s="1"/>
-  <c r="A25" i="1" s="1"/>
-  <c r="A26" i="1" s="1"/>
-  <c r="A27" i="1" s="1"/>
-  <c r="A28" i="1" s="1"/>
-  <c r="A29" i="1" s="1"/>
-  <c r="A30" i="1" s="1"/>
-  <c r="A31" i="1" s="1"/>
-  <c r="A32" i="1" s="1"/>
-  <c r="A33" i="1" s="1"/>
-  <c r="A34" i="1" s="1"/>
-  <c r="A35" i="1" s="1"/>
-  <c r="A36" i="1" s="1"/>
-  <c r="A37" i="1" s="1"/>
-  <c r="A38" i="1" s="1"/>
-  <c r="A39" i="1" s="1"/>
-  <c r="A40" i="1" s="1"/>
-  <c r="A41" i="1" s="1"/>
-  <c r="A42" i="1" s="1"/>
-  <c r="A43" i="1" s="1"/>
-  <c r="A44" i="1" s="1"/>
-  <c r="A45" i="1" s="1"/>
-  <c r="A46" i="1" s="1"/>
-  <c r="A47" i="1" s="1"/>
-  <c r="A48" i="1" s="1"/>
-  <c r="A49" i="1" s="1"/>
-  <c r="A50" i="1" s="1"/>
-  <c r="A51" i="1" s="1"/>
-  <c r="A52" i="1" s="1"/>
-  <c r="A53" i="1" s="1"/>
-  <c r="A54" i="1" s="1"/>
-  <c r="A55" i="1" s="1"/>
-  <c r="A56" i="1" s="1"/>
-  <c r="A57" i="1" s="1"/>
-  <c r="A58" i="1" s="1"/>
-  <c r="A59" i="1" s="1"/>
-  <c r="A60" i="1" s="1"/>
-  <c r="A61" i="1" s="1"/>
-  <c r="A62" i="1" s="1"/>
-  <c r="A63" i="1" s="1"/>
-  <c r="A64" i="1" s="1"/>
-  <c r="A65" i="1" s="1"/>
-  <c r="A66" i="1" s="1"/>
-  <c r="A67" i="1" s="1"/>
-  <c r="A68" i="1" s="1"/>
-  <c r="A69" i="1" s="1"/>
-  <c r="A70" i="1" s="1"/>
-  <c r="A71" i="1" s="1"/>
-  <c r="A72" i="1" s="1"/>
-  <c r="A73" i="1" s="1"/>
-  <c r="A74" i="1" s="1"/>
-  <c r="A75" i="1" s="1"/>
-  <c r="A76" i="1" s="1"/>
-  <c r="A77" i="1" s="1"/>
-  <c r="A78" i="1" s="1"/>
-  <c r="A79" i="1" s="1"/>
-  <c r="A80" i="1" s="1"/>
-  <c r="A81" i="1" s="1"/>
-  <c r="A82" i="1" s="1"/>
-  <c r="A83" i="1" s="1"/>
-  <c r="A84" i="1" s="1"/>
-  <c r="A85" i="1" s="1"/>
-  <c r="A86" i="1" s="1"/>
-  <c r="A87" i="1" s="1"/>
-  <c r="A88" i="1" s="1"/>
-  <c r="A89" i="1" s="1"/>
-  <c r="A90" i="1" s="1"/>
-  <c r="A91" i="1" s="1"/>
-  <c r="A92" i="1" s="1"/>
-  <c r="A93" i="1" s="1"/>
-  <c r="A94" i="1" s="1"/>
-  <c r="A95" i="1" s="1"/>
-  <c r="A96" i="1" s="1"/>
-  <c r="A97" i="1" s="1"/>
-  <c r="A98" i="1" s="1"/>
-  <c r="A99" i="1" s="1"/>
-  <c r="A100" i="1" s="1"/>
-  <c r="A101" i="1" s="1"/>
-  <c r="A102" i="1" s="1"/>
-  <c r="A103" i="1" s="1"/>
-  <c r="A104" i="1" s="1"/>
-  <c r="A105" i="1" s="1"/>
-  <c r="A106" i="1" s="1"/>
-  <c r="A107" i="1" s="1"/>
-  <c r="A108" i="1" s="1"/>
-  <c r="A109" i="1" s="1"/>
-  <c r="A110" i="1" s="1"/>
-  <c r="A111" i="1" s="1"/>
-  <c r="A112" i="1" s="1"/>
-  <c r="A113" i="1" s="1"/>
-  <c r="A114" i="1" s="1"/>
-  <c r="A115" i="1" s="1"/>
-  <c r="A116" i="1" s="1"/>
-  <c r="A117" i="1" s="1"/>
-  <c r="A118" i="1" s="1"/>
-  <c r="A119" i="1" s="1"/>
-  <c r="A120" i="1" s="1"/>
-  <c r="A121" i="1" s="1"/>
-  <c r="A122" i="1" s="1"/>
-  <c r="A123" i="1" s="1"/>
-  <c r="A124" i="1" s="1"/>
-  <c r="A125" i="1" s="1"/>
-  <c r="A126" i="1" s="1"/>
-  <c r="A127" i="1" s="1"/>
-  <c r="A128" i="1" s="1"/>
-  <c r="A129" i="1" s="1"/>
-  <c r="A130" i="1" s="1"/>
-  <c r="A131" i="1" s="1"/>
-  <c r="A132" i="1" s="1"/>
-  <c r="A133" i="1" s="1"/>
-  <c r="A134" i="1" s="1"/>
-  <c r="A135" i="1" s="1"/>
-  <c r="A136" i="1" s="1"/>
-  <c r="A137" i="1" s="1"/>
-  <c r="A138" i="1" s="1"/>
-  <c r="A139" i="1" s="1"/>
-  <c r="A140" i="1" s="1"/>
-  <c r="A141" i="1" s="1"/>
-  <c r="A142" i="1" s="1"/>
-  <c r="A143" i="1" s="1"/>
-  <c r="A144" i="1" s="1"/>
-  <c r="A145" i="1" s="1"/>
-  <c r="A146" i="1" s="1"/>
-  <c r="A147" i="1" s="1"/>
-  <c r="A148" i="1" s="1"/>
-  <c r="A149" i="1" s="1"/>
-  <c r="A150" i="1" s="1"/>
-  <c r="A151" i="1" s="1"/>
-  <c r="A152" i="1" s="1"/>
-  <c r="A153" i="1" s="1"/>
-  <c r="A154" i="1" s="1"/>
-  <c r="A155" i="1" s="1"/>
-  <c r="A156" i="1" s="1"/>
-  <c r="A157" i="1" s="1"/>
-  <c r="A158" i="1" s="1"/>
-  <c r="A159" i="1" s="1"/>
-  <c r="A160" i="1" s="1"/>
-  <c r="A161" i="1" s="1"/>
-  <c r="A162" i="1" s="1"/>
-  <c r="A163" i="1" s="1"/>
-  <c r="A164" i="1" s="1"/>
-  <c r="A165" i="1" s="1"/>
-  <c r="A166" i="1" s="1"/>
-  <c r="A167" i="1" s="1"/>
-  <c r="A168" i="1" s="1"/>
-  <c r="A169" i="1" s="1"/>
-  <c r="A170" i="1" s="1"/>
-  <c r="A171" i="1" s="1"/>
-  <c r="A172" i="1" s="1"/>
-  <c r="A173" i="1" s="1"/>
-  <c r="A174" i="1" s="1"/>
-  <c r="A175" i="1" s="1"/>
-  <c r="A176" i="1" s="1"/>
-  <c r="A177" i="1" s="1"/>
-  <c r="A178" i="1" s="1"/>
-  <c r="A179" i="1" s="1"/>
-  <c r="A180" i="1" s="1"/>
-  <c r="A181" i="1" s="1"/>
-  <c r="A182" i="1" s="1"/>
-  <c r="A183" i="1" s="1"/>
-  <c r="A184" i="1" s="1"/>
-  <c r="A185" i="1" s="1"/>
-  <c r="A186" i="1" s="1"/>
-  <c r="A187" i="1" s="1"/>
-  <c r="A188" i="1" s="1"/>
-  <c r="A189" i="1" s="1"/>
-  <c r="A190" i="1" s="1"/>
-  <c r="A191" i="1" s="1"/>
-  <c r="A192" i="1" s="1"/>
-  <c r="A193" i="1" s="1"/>
-  <c r="A194" i="1" s="1"/>
-  <c r="A195" i="1" s="1"/>
-  <c r="A196" i="1" s="1"/>
-  <c r="A197" i="1" s="1"/>
-  <c r="A198" i="1" s="1"/>
-</calcChain>
-</file>
-
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="860">
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="864">
   <si>
     <t>Number</t>
   </si>
@@ -2864,10 +2658,22 @@
   <si>
     <t>When surrounded by conformity, how much of yourself are you willing to keep visible?</t>
   </si>
+  <si>
+    <t>The Fifth Apple</t>
+  </si>
+  <si>
+    <t>In a tranquil orchard bathed in soft evening light, an elderly photographer stands at the edge of the frame, camera raised, documenting an extraordinary encounter across time. Beneath a sprawling apple tree sits Sir Isaac Newton, dressed in period clothing and holding an open book, his gaze lifted toward a single red apple hanging above him. Several fallen apples scatter the grass around him, while the modern photographer—part observer, part intruder—appears to capture the very instant before revelation strikes. The composition juxtaposes centuries through costume, posture, and technology, blending pastoral serenity with subtle temporal dissonance. The warm cinematic lighting and carefully balanced framing create the feeling of a historical memory interrupted by contemporary consciousness.</t>
+  </si>
+  <si>
+    <t>The image explores the fragile boundary between observation and discovery, suggesting that every great revelation depends not only on the thinker, but also on the witness who frames the moment. By inserting the modern photographer into Newton’s iconic scene, the work transforms a familiar scientific myth into a meditation on humanity’s endless desire to revisit, reinterpret, and preserve the origins of knowledge. The “fifth apple” implied by the title may symbolize the unseen or undocumented layer of history—the observer outside the narrative who nevertheless shapes its meaning. The scattered apples evoke repetition and inevitability, while the suspended apple above Newton represents the moment before understanding crystallizes. The photographer’s presence also introduces questions about authenticity, memory, and artistic intervention: are we documenting history, recreating it, or subtly rewriting it through the act of looking? Beneath its quiet humor lies a deeper reflection on time travel, intellectual inheritance, and the modern compulsion to stand inside legendary moments rather than merely study them from afar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At what point does repetition become revelation? </t>
+  </si>
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
@@ -2961,7 +2767,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -3244,40 +3050,9 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Programming\MyCellphoeApp\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77390DFE-F443-404A-BA9D-A23DC4070CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G215"/>
+  <dimension ref="A1:G216"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -7772,6 +7547,23 @@
         <v>46163</v>
       </c>
     </row>
+    <row r="216" spans="1:6" ht="213.75" x14ac:dyDescent="0.2">
+      <c r="B216" t="s">
+        <v>860</v>
+      </c>
+      <c r="C216" s="1" t="s">
+        <v>861</v>
+      </c>
+      <c r="D216" s="1" t="s">
+        <v>862</v>
+      </c>
+      <c r="E216" t="s">
+        <v>863</v>
+      </c>
+      <c r="F216" s="5">
+        <v>46165</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Add An Image Is Born update
</commit_message>
<xml_diff>
--- a/data/image_data.xlsx
+++ b/data/image_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Programming\MyCellphoeApp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB73146-E38F-40B7-86E7-B3B4E16CE8DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E09FC17-2924-4C98-8BE2-DB933F6BEA55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="864">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="868">
   <si>
     <t>Number</t>
   </si>
@@ -2669,6 +2669,18 @@
   </si>
   <si>
     <t xml:space="preserve">At what point does repetition become revelation? </t>
+  </si>
+  <si>
+    <t>An Image Is Born</t>
+  </si>
+  <si>
+    <t>An Image Is Born presents a dark, dreamlike interior seen from an impossible overhead perspective, as if the viewer is looking down into a room that has partially opened into outer space. On the left, an elderly bald man in a red shirt sleeps in bed beneath a heavy blanket, his hands folded calmly over his body, illuminated by a small bedside lamp. At the bottom center, the same man appears again, seated at a computer desk, seen from above, working on an image displayed on the monitor. Above him, the ceiling or upper wall seems to have ruptured, transforming into a vast cosmic landscape of stars, a ringed planet, a luminous spiral galaxy, and a rocky lunar-like surface. A third version of the man, again in a red shirt, sits on this cosmic terrain, gazing silently into the galactic distance. The room itself is dense, shadowy, and cluttered with framed pictures, books, devices, drawers, clocks, and studio-like objects, giving the impression of a private creative chamber where domestic reality, digital labor, and visionary imagination coexist in a single theatrical space.</t>
+  </si>
+  <si>
+    <t>The image powerfully stages the birth of an artwork as a layered process moving between sleep, craft, and metaphysical projection. The sleeping figure suggests the unconscious source of creation: the dream, the buried image, the private psychic reservoir from which visual ideas emerge. The seated figure at the computer represents the disciplined maker, the technician, the editor, the conscious artist who translates dream-material into constructed form. The third figure, sitting on the cosmic surface, becomes the inner traveler or visionary self—the one who has already crossed from the ordinary room into the imagined universe. The rupture between bedroom and galaxy is especially significant: creation is not shown as simple inspiration, but as a break in the ceiling of reality, an opening through which the finite human self encounters immensity. The repeated red shirt links the three selves into one continuous identity, while their separate positions imply three states of being: dreamer, maker, and wanderer. At its deepest level, the work is a self-portrait of artistic consciousness itself: the elderly artist’s body remains in the small room, but his imagination expands into astronomical scale, turning solitude, aging, and night-work into a private act of cosmic exploration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What part of you travels farthest when the body remains asleep at home? </t>
   </si>
 </sst>
 </file>
@@ -2717,21 +2729,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2745,11 +2748,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3052,13 +3057,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G216"/>
+  <dimension ref="A1:G217"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="34.25" customWidth="1"/>
     <col min="3" max="5" width="70" customWidth="1"/>
-    <col min="6" max="6" width="14" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -3077,7 +3082,7 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
     </row>
@@ -3097,7 +3102,7 @@
       <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="9">
         <v>45280</v>
       </c>
     </row>
@@ -3118,7 +3123,7 @@
       <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="9">
         <v>45199</v>
       </c>
     </row>
@@ -3139,7 +3144,7 @@
       <c r="E4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="9">
         <v>45057</v>
       </c>
     </row>
@@ -3160,7 +3165,7 @@
       <c r="E5" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="9">
         <v>45057</v>
       </c>
     </row>
@@ -3181,7 +3186,7 @@
       <c r="E6" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="9">
         <v>44799</v>
       </c>
     </row>
@@ -3202,7 +3207,7 @@
       <c r="E7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="9">
         <v>45678</v>
       </c>
     </row>
@@ -3223,7 +3228,7 @@
       <c r="E8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="9">
         <v>45182</v>
       </c>
     </row>
@@ -3244,7 +3249,7 @@
       <c r="E9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="9">
         <v>45057</v>
       </c>
     </row>
@@ -3265,7 +3270,7 @@
       <c r="E10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="9">
         <v>45265</v>
       </c>
     </row>
@@ -3286,7 +3291,7 @@
       <c r="E11" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="9">
         <v>45606</v>
       </c>
     </row>
@@ -3307,7 +3312,7 @@
       <c r="E12" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="9">
         <v>45390</v>
       </c>
     </row>
@@ -3328,7 +3333,7 @@
       <c r="E13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="9">
         <v>45706</v>
       </c>
     </row>
@@ -3349,7 +3354,7 @@
       <c r="E14" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="9">
         <v>45057</v>
       </c>
     </row>
@@ -3370,7 +3375,7 @@
       <c r="E15" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="9">
         <v>45052</v>
       </c>
     </row>
@@ -3391,7 +3396,7 @@
       <c r="E16" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="9">
         <v>45058</v>
       </c>
     </row>
@@ -3412,7 +3417,7 @@
       <c r="E17" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="9">
         <v>44638</v>
       </c>
     </row>
@@ -3433,7 +3438,7 @@
       <c r="E18" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="9">
         <v>45746</v>
       </c>
     </row>
@@ -3454,7 +3459,7 @@
       <c r="E19" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="9">
         <v>45384</v>
       </c>
     </row>
@@ -3475,7 +3480,7 @@
       <c r="E20" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="9">
         <v>45470</v>
       </c>
     </row>
@@ -3496,7 +3501,7 @@
       <c r="E21" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="9">
         <v>45057</v>
       </c>
     </row>
@@ -3517,7 +3522,7 @@
       <c r="E22" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="9">
         <v>45703</v>
       </c>
     </row>
@@ -3538,7 +3543,7 @@
       <c r="E23" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F23" s="9">
         <v>45054</v>
       </c>
     </row>
@@ -3559,7 +3564,7 @@
       <c r="E24" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="9">
         <v>43608</v>
       </c>
     </row>
@@ -3580,7 +3585,7 @@
       <c r="E25" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="F25" s="3">
+      <c r="F25" s="9">
         <v>45332</v>
       </c>
     </row>
@@ -3601,7 +3606,7 @@
       <c r="E26" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="F26" s="3">
+      <c r="F26" s="9">
         <v>45296</v>
       </c>
     </row>
@@ -3622,7 +3627,7 @@
       <c r="E27" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="F27" s="3">
+      <c r="F27" s="9">
         <v>45061</v>
       </c>
     </row>
@@ -3643,7 +3648,7 @@
       <c r="E28" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="F28" s="3">
+      <c r="F28" s="9">
         <v>45145</v>
       </c>
     </row>
@@ -3664,7 +3669,7 @@
       <c r="E29" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F29" s="3">
+      <c r="F29" s="9">
         <v>45157</v>
       </c>
     </row>
@@ -3685,7 +3690,7 @@
       <c r="E30" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="9">
         <v>45314</v>
       </c>
     </row>
@@ -3706,7 +3711,7 @@
       <c r="E31" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="F31" s="3">
+      <c r="F31" s="9">
         <v>45059</v>
       </c>
     </row>
@@ -3727,7 +3732,7 @@
       <c r="E32" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="F32" s="3">
+      <c r="F32" s="9">
         <v>45472</v>
       </c>
     </row>
@@ -3748,7 +3753,7 @@
       <c r="E33" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F33" s="3">
+      <c r="F33" s="9">
         <v>45720</v>
       </c>
     </row>
@@ -3769,7 +3774,7 @@
       <c r="E34" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="F34" s="3">
+      <c r="F34" s="9">
         <v>45448</v>
       </c>
     </row>
@@ -3790,7 +3795,7 @@
       <c r="E35" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F35" s="3">
+      <c r="F35" s="9">
         <v>45449</v>
       </c>
     </row>
@@ -3811,7 +3816,7 @@
       <c r="E36" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="F36" s="3">
+      <c r="F36" s="9">
         <v>45048</v>
       </c>
     </row>
@@ -3832,7 +3837,7 @@
       <c r="E37" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="F37" s="3">
+      <c r="F37" s="9">
         <v>45660</v>
       </c>
     </row>
@@ -3853,7 +3858,7 @@
       <c r="E38" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F38" s="3">
+      <c r="F38" s="9">
         <v>45057</v>
       </c>
     </row>
@@ -3874,7 +3879,7 @@
       <c r="E39" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="F39" s="3">
+      <c r="F39" s="9">
         <v>45301</v>
       </c>
     </row>
@@ -3895,7 +3900,7 @@
       <c r="E40" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F40" s="9">
         <v>44921</v>
       </c>
     </row>
@@ -3916,7 +3921,7 @@
       <c r="E41" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="F41" s="3">
+      <c r="F41" s="9">
         <v>45042</v>
       </c>
     </row>
@@ -3937,7 +3942,7 @@
       <c r="E42" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="F42" s="3">
+      <c r="F42" s="9">
         <v>45056</v>
       </c>
     </row>
@@ -3958,7 +3963,7 @@
       <c r="E43" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="F43" s="3">
+      <c r="F43" s="9">
         <v>45472</v>
       </c>
     </row>
@@ -3979,7 +3984,7 @@
       <c r="E44" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F44" s="3">
+      <c r="F44" s="9">
         <v>44819</v>
       </c>
     </row>
@@ -4000,7 +4005,7 @@
       <c r="E45" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="F45" s="3">
+      <c r="F45" s="9">
         <v>45366</v>
       </c>
     </row>
@@ -4021,7 +4026,7 @@
       <c r="E46" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="F46" s="3">
+      <c r="F46" s="9">
         <v>45135</v>
       </c>
     </row>
@@ -4042,7 +4047,7 @@
       <c r="E47" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="F47" s="3">
+      <c r="F47" s="9">
         <v>45729</v>
       </c>
     </row>
@@ -4063,7 +4068,7 @@
       <c r="E48" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="F48" s="3">
+      <c r="F48" s="9">
         <v>45772</v>
       </c>
     </row>
@@ -4084,7 +4089,7 @@
       <c r="E49" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="F49" s="3">
+      <c r="F49" s="9">
         <v>45749</v>
       </c>
     </row>
@@ -4105,7 +4110,7 @@
       <c r="E50" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="F50" s="3">
+      <c r="F50" s="9">
         <v>45744</v>
       </c>
     </row>
@@ -4126,7 +4131,7 @@
       <c r="E51" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="F51" s="3">
+      <c r="F51" s="9">
         <v>45573</v>
       </c>
     </row>
@@ -4147,7 +4152,7 @@
       <c r="E52" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="F52" s="3">
+      <c r="F52" s="9">
         <v>45541</v>
       </c>
     </row>
@@ -4168,7 +4173,7 @@
       <c r="E53" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="F53" s="3">
+      <c r="F53" s="9">
         <v>44630</v>
       </c>
     </row>
@@ -4189,7 +4194,7 @@
       <c r="E54" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="F54" s="3">
+      <c r="F54" s="9">
         <v>45610</v>
       </c>
     </row>
@@ -4210,7 +4215,7 @@
       <c r="E55" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="F55" s="3">
+      <c r="F55" s="9">
         <v>45770</v>
       </c>
     </row>
@@ -4231,7 +4236,7 @@
       <c r="E56" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="F56" s="3">
+      <c r="F56" s="9">
         <v>45334</v>
       </c>
     </row>
@@ -4252,7 +4257,7 @@
       <c r="E57" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="F57" s="3">
+      <c r="F57" s="9">
         <v>45334</v>
       </c>
     </row>
@@ -4273,7 +4278,7 @@
       <c r="E58" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="F58" s="3">
+      <c r="F58" s="9">
         <v>45621</v>
       </c>
     </row>
@@ -4294,7 +4299,7 @@
       <c r="E59" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="F59" s="3">
+      <c r="F59" s="9">
         <v>45062</v>
       </c>
     </row>
@@ -4315,7 +4320,7 @@
       <c r="E60" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="F60" s="3">
+      <c r="F60" s="9">
         <v>45157</v>
       </c>
     </row>
@@ -4336,7 +4341,7 @@
       <c r="E61" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="F61" s="3">
+      <c r="F61" s="9">
         <v>45473</v>
       </c>
     </row>
@@ -4357,7 +4362,7 @@
       <c r="E62" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="F62" s="4"/>
+      <c r="F62" s="10"/>
     </row>
     <row r="63" spans="1:6" ht="128.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2">
@@ -4376,7 +4381,7 @@
       <c r="E63" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="F63" s="3">
+      <c r="F63" s="9">
         <v>45155</v>
       </c>
     </row>
@@ -4397,7 +4402,7 @@
       <c r="E64" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="F64" s="3">
+      <c r="F64" s="9">
         <v>45052</v>
       </c>
     </row>
@@ -4418,7 +4423,7 @@
       <c r="E65" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="F65" s="3">
+      <c r="F65" s="9">
         <v>45341</v>
       </c>
     </row>
@@ -4439,7 +4444,7 @@
       <c r="E66" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="F66" s="3">
+      <c r="F66" s="9">
         <v>45555</v>
       </c>
     </row>
@@ -4460,7 +4465,7 @@
       <c r="E67" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="F67" s="3">
+      <c r="F67" s="9">
         <v>45054</v>
       </c>
     </row>
@@ -4481,7 +4486,7 @@
       <c r="E68" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="F68" s="3">
+      <c r="F68" s="9">
         <v>45057</v>
       </c>
     </row>
@@ -4502,7 +4507,7 @@
       <c r="E69" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="F69" s="3">
+      <c r="F69" s="9">
         <v>45042</v>
       </c>
     </row>
@@ -4523,7 +4528,7 @@
       <c r="E70" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="F70" s="3">
+      <c r="F70" s="9">
         <v>45046</v>
       </c>
     </row>
@@ -4544,7 +4549,7 @@
       <c r="E71" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="F71" s="3">
+      <c r="F71" s="9">
         <v>45063</v>
       </c>
     </row>
@@ -4565,7 +4570,7 @@
       <c r="E72" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="F72" s="3">
+      <c r="F72" s="9">
         <v>45687</v>
       </c>
     </row>
@@ -4574,7 +4579,7 @@
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="B73" s="7" t="s">
+      <c r="B73" s="4" t="s">
         <v>290</v>
       </c>
       <c r="C73" s="1" t="s">
@@ -4586,7 +4591,7 @@
       <c r="E73" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F73" s="3">
+      <c r="F73" s="9">
         <v>45488</v>
       </c>
     </row>
@@ -4607,7 +4612,7 @@
       <c r="E74" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="F74" s="3">
+      <c r="F74" s="9">
         <v>45054</v>
       </c>
     </row>
@@ -4628,7 +4633,7 @@
       <c r="E75" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="F75" s="3">
+      <c r="F75" s="9">
         <v>45448</v>
       </c>
     </row>
@@ -4649,7 +4654,7 @@
       <c r="E76" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="F76" s="3">
+      <c r="F76" s="9">
         <v>45766</v>
       </c>
     </row>
@@ -4670,7 +4675,7 @@
       <c r="E77" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="F77" s="3">
+      <c r="F77" s="9">
         <v>45675</v>
       </c>
     </row>
@@ -4691,7 +4696,7 @@
       <c r="E78" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="F78" s="3">
+      <c r="F78" s="9">
         <v>45312</v>
       </c>
     </row>
@@ -4712,7 +4717,7 @@
       <c r="E79" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="F79" s="3">
+      <c r="F79" s="9">
         <v>45051</v>
       </c>
     </row>
@@ -4733,7 +4738,7 @@
       <c r="E80" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="F80" s="3">
+      <c r="F80" s="9">
         <v>45053</v>
       </c>
     </row>
@@ -4754,7 +4759,7 @@
       <c r="E81" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="F81" s="3">
+      <c r="F81" s="9">
         <v>45092</v>
       </c>
     </row>
@@ -4775,7 +4780,7 @@
       <c r="E82" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="F82" s="3">
+      <c r="F82" s="9">
         <v>45721</v>
       </c>
     </row>
@@ -4796,7 +4801,7 @@
       <c r="E83" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="F83" s="3">
+      <c r="F83" s="9">
         <v>45419</v>
       </c>
     </row>
@@ -4817,7 +4822,7 @@
       <c r="E84" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="F84" s="3">
+      <c r="F84" s="9">
         <v>45419</v>
       </c>
     </row>
@@ -4838,7 +4843,7 @@
       <c r="E85" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="F85" s="3">
+      <c r="F85" s="9">
         <v>45146</v>
       </c>
     </row>
@@ -4859,7 +4864,7 @@
       <c r="E86" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="F86" s="3">
+      <c r="F86" s="9">
         <v>45453</v>
       </c>
     </row>
@@ -4880,7 +4885,7 @@
       <c r="E87" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="F87" s="3">
+      <c r="F87" s="9">
         <v>45479</v>
       </c>
     </row>
@@ -4901,7 +4906,7 @@
       <c r="E88" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F88" s="3">
+      <c r="F88" s="9">
         <v>45324</v>
       </c>
     </row>
@@ -4922,7 +4927,7 @@
       <c r="E89" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="F89" s="3">
+      <c r="F89" s="9">
         <v>45045</v>
       </c>
     </row>
@@ -4943,7 +4948,7 @@
       <c r="E90" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="F90" s="3">
+      <c r="F90" s="9">
         <v>45673</v>
       </c>
     </row>
@@ -4964,7 +4969,7 @@
       <c r="E91" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="F91" s="3">
+      <c r="F91" s="9">
         <v>45296</v>
       </c>
     </row>
@@ -4985,7 +4990,7 @@
       <c r="E92" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="F92" s="3">
+      <c r="F92" s="9">
         <v>44692</v>
       </c>
     </row>
@@ -5006,7 +5011,7 @@
       <c r="E93" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="F93" s="4"/>
+      <c r="F93" s="10"/>
     </row>
     <row r="94" spans="1:6" ht="128.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="2">
@@ -5025,7 +5030,7 @@
       <c r="E94" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="F94" s="3">
+      <c r="F94" s="9">
         <v>45058</v>
       </c>
     </row>
@@ -5046,7 +5051,7 @@
       <c r="E95" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="F95" s="3">
+      <c r="F95" s="9">
         <v>45695</v>
       </c>
     </row>
@@ -5067,7 +5072,7 @@
       <c r="E96" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="F96" s="3">
+      <c r="F96" s="9">
         <v>45193</v>
       </c>
     </row>
@@ -5088,7 +5093,7 @@
       <c r="E97" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="F97" s="3">
+      <c r="F97" s="9">
         <v>45494</v>
       </c>
     </row>
@@ -5109,7 +5114,7 @@
       <c r="E98" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="F98" s="3">
+      <c r="F98" s="9">
         <v>45691</v>
       </c>
     </row>
@@ -5130,7 +5135,7 @@
       <c r="E99" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="F99" s="3">
+      <c r="F99" s="9">
         <v>45671</v>
       </c>
     </row>
@@ -5151,7 +5156,7 @@
       <c r="E100" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="F100" s="3">
+      <c r="F100" s="9">
         <v>45019</v>
       </c>
     </row>
@@ -5172,7 +5177,7 @@
       <c r="E101" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="F101" s="3">
+      <c r="F101" s="9">
         <v>45661</v>
       </c>
     </row>
@@ -5193,7 +5198,7 @@
       <c r="E102" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="F102" s="3">
+      <c r="F102" s="9">
         <v>45236</v>
       </c>
     </row>
@@ -5214,7 +5219,7 @@
       <c r="E103" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="F103" s="3">
+      <c r="F103" s="9">
         <v>45241</v>
       </c>
     </row>
@@ -5235,7 +5240,7 @@
       <c r="E104" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="F104" s="3">
+      <c r="F104" s="9">
         <v>45260</v>
       </c>
     </row>
@@ -5256,7 +5261,7 @@
       <c r="E105" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="F105" s="3">
+      <c r="F105" s="9">
         <v>45579</v>
       </c>
     </row>
@@ -5277,7 +5282,7 @@
       <c r="E106" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="F106" s="3">
+      <c r="F106" s="9">
         <v>45057</v>
       </c>
     </row>
@@ -5298,7 +5303,7 @@
       <c r="E107" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="F107" s="3">
+      <c r="F107" s="9">
         <v>45704</v>
       </c>
     </row>
@@ -5319,7 +5324,7 @@
       <c r="E108" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="F108" s="3">
+      <c r="F108" s="9">
         <v>45634</v>
       </c>
     </row>
@@ -5340,7 +5345,7 @@
       <c r="E109" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="F109" s="3">
+      <c r="F109" s="9">
         <v>45064</v>
       </c>
     </row>
@@ -5361,7 +5366,7 @@
       <c r="E110" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="F110" s="3">
+      <c r="F110" s="9">
         <v>45064</v>
       </c>
     </row>
@@ -5382,7 +5387,7 @@
       <c r="E111" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="F111" s="3">
+      <c r="F111" s="9">
         <v>45248</v>
       </c>
     </row>
@@ -5403,7 +5408,7 @@
       <c r="E112" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="F112" s="3">
+      <c r="F112" s="9">
         <v>45259</v>
       </c>
     </row>
@@ -5424,7 +5429,7 @@
       <c r="E113" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="F113" s="3">
+      <c r="F113" s="9">
         <v>45313</v>
       </c>
     </row>
@@ -5445,7 +5450,7 @@
       <c r="E114" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="F114" s="3">
+      <c r="F114" s="9">
         <v>45615</v>
       </c>
     </row>
@@ -5466,7 +5471,7 @@
       <c r="E115" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="F115" s="3">
+      <c r="F115" s="9">
         <v>45621</v>
       </c>
     </row>
@@ -5487,7 +5492,7 @@
       <c r="E116" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="F116" s="3">
+      <c r="F116" s="9">
         <v>45186</v>
       </c>
     </row>
@@ -5508,7 +5513,7 @@
       <c r="E117" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="F117" s="3">
+      <c r="F117" s="9">
         <v>45130</v>
       </c>
     </row>
@@ -5529,7 +5534,7 @@
       <c r="E118" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="F118" s="3">
+      <c r="F118" s="9">
         <v>45227</v>
       </c>
     </row>
@@ -5550,7 +5555,7 @@
       <c r="E119" s="1" t="s">
         <v>477</v>
       </c>
-      <c r="F119" s="3">
+      <c r="F119" s="9">
         <v>45661</v>
       </c>
     </row>
@@ -5571,7 +5576,7 @@
       <c r="E120" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="F120" s="3">
+      <c r="F120" s="9">
         <v>45042</v>
       </c>
     </row>
@@ -5592,7 +5597,7 @@
       <c r="E121" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="F121" s="3">
+      <c r="F121" s="9">
         <v>45452</v>
       </c>
     </row>
@@ -5613,7 +5618,7 @@
       <c r="E122" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="F122" s="3">
+      <c r="F122" s="9">
         <v>45640</v>
       </c>
     </row>
@@ -5634,7 +5639,7 @@
       <c r="E123" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="F123" s="3">
+      <c r="F123" s="9">
         <v>45117</v>
       </c>
     </row>
@@ -5655,7 +5660,7 @@
       <c r="E124" s="1" t="s">
         <v>497</v>
       </c>
-      <c r="F124" s="3">
+      <c r="F124" s="9">
         <v>45194</v>
       </c>
     </row>
@@ -5676,7 +5681,7 @@
       <c r="E125" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="F125" s="4"/>
+      <c r="F125" s="10"/>
     </row>
     <row r="126" spans="1:6" ht="128.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="2">
@@ -5695,7 +5700,7 @@
       <c r="E126" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="F126" s="3">
+      <c r="F126" s="9">
         <v>45685</v>
       </c>
     </row>
@@ -5716,7 +5721,7 @@
       <c r="E127" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="F127" s="3">
+      <c r="F127" s="9">
         <v>45476</v>
       </c>
     </row>
@@ -5737,7 +5742,7 @@
       <c r="E128" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="F128" s="3">
+      <c r="F128" s="9">
         <v>45659</v>
       </c>
     </row>
@@ -5758,7 +5763,7 @@
       <c r="E129" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="F129" s="3">
+      <c r="F129" s="9">
         <v>45216</v>
       </c>
     </row>
@@ -5779,7 +5784,7 @@
       <c r="E130" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="F130" s="4"/>
+      <c r="F130" s="10"/>
     </row>
     <row r="131" spans="1:6" ht="185.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="2">
@@ -5798,7 +5803,7 @@
       <c r="E131" s="1" t="s">
         <v>525</v>
       </c>
-      <c r="F131" s="3">
+      <c r="F131" s="9">
         <v>45720</v>
       </c>
     </row>
@@ -5819,7 +5824,7 @@
       <c r="E132" s="1" t="s">
         <v>529</v>
       </c>
-      <c r="F132" s="3">
+      <c r="F132" s="9">
         <v>45720</v>
       </c>
     </row>
@@ -5840,7 +5845,7 @@
       <c r="E133" s="1" t="s">
         <v>533</v>
       </c>
-      <c r="F133" s="3">
+      <c r="F133" s="9">
         <v>45699</v>
       </c>
     </row>
@@ -5861,7 +5866,7 @@
       <c r="E134" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="F134" s="3">
+      <c r="F134" s="9">
         <v>45462</v>
       </c>
     </row>
@@ -5882,7 +5887,7 @@
       <c r="E135" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="F135" s="3">
+      <c r="F135" s="9">
         <v>45057</v>
       </c>
     </row>
@@ -5903,7 +5908,7 @@
       <c r="E136" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="F136" s="3">
+      <c r="F136" s="9">
         <v>45484</v>
       </c>
     </row>
@@ -5924,7 +5929,7 @@
       <c r="E137" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="F137" s="3">
+      <c r="F137" s="9">
         <v>45061</v>
       </c>
     </row>
@@ -5945,7 +5950,7 @@
       <c r="E138" s="1" t="s">
         <v>552</v>
       </c>
-      <c r="F138" s="3">
+      <c r="F138" s="9">
         <v>45098</v>
       </c>
     </row>
@@ -5966,7 +5971,7 @@
       <c r="E139" s="1" t="s">
         <v>556</v>
       </c>
-      <c r="F139" s="3">
+      <c r="F139" s="9">
         <v>45053</v>
       </c>
     </row>
@@ -5987,7 +5992,7 @@
       <c r="E140" s="1" t="s">
         <v>560</v>
       </c>
-      <c r="F140" s="3">
+      <c r="F140" s="9">
         <v>45591</v>
       </c>
     </row>
@@ -6008,7 +6013,7 @@
       <c r="E141" s="1" t="s">
         <v>564</v>
       </c>
-      <c r="F141" s="3">
+      <c r="F141" s="9">
         <v>45591</v>
       </c>
     </row>
@@ -6029,7 +6034,7 @@
       <c r="E142" s="1" t="s">
         <v>568</v>
       </c>
-      <c r="F142" s="3">
+      <c r="F142" s="9">
         <v>45588</v>
       </c>
     </row>
@@ -6050,7 +6055,7 @@
       <c r="E143" s="1" t="s">
         <v>572</v>
       </c>
-      <c r="F143" s="3">
+      <c r="F143" s="9">
         <v>45096</v>
       </c>
     </row>
@@ -6071,7 +6076,7 @@
       <c r="E144" s="1" t="s">
         <v>576</v>
       </c>
-      <c r="F144" s="3">
+      <c r="F144" s="9">
         <v>45348</v>
       </c>
     </row>
@@ -6092,7 +6097,7 @@
       <c r="E145" s="1" t="s">
         <v>580</v>
       </c>
-      <c r="F145" s="3">
+      <c r="F145" s="9">
         <v>45604</v>
       </c>
     </row>
@@ -6113,7 +6118,7 @@
       <c r="E146" s="1" t="s">
         <v>584</v>
       </c>
-      <c r="F146" s="3">
+      <c r="F146" s="9">
         <v>45479</v>
       </c>
     </row>
@@ -6134,7 +6139,7 @@
       <c r="E147" s="1" t="s">
         <v>588</v>
       </c>
-      <c r="F147" s="3">
+      <c r="F147" s="9">
         <v>45450</v>
       </c>
     </row>
@@ -6155,7 +6160,7 @@
       <c r="E148" s="1" t="s">
         <v>592</v>
       </c>
-      <c r="F148" s="3">
+      <c r="F148" s="9">
         <v>45668</v>
       </c>
     </row>
@@ -6176,7 +6181,7 @@
       <c r="E149" s="1" t="s">
         <v>596</v>
       </c>
-      <c r="F149" s="3">
+      <c r="F149" s="9">
         <v>45780</v>
       </c>
     </row>
@@ -6197,7 +6202,7 @@
       <c r="E150" s="1" t="s">
         <v>600</v>
       </c>
-      <c r="F150" s="3">
+      <c r="F150" s="9">
         <v>45784</v>
       </c>
     </row>
@@ -6218,7 +6223,7 @@
       <c r="E151" s="1" t="s">
         <v>604</v>
       </c>
-      <c r="F151" s="3">
+      <c r="F151" s="9">
         <v>45785</v>
       </c>
     </row>
@@ -6239,7 +6244,7 @@
       <c r="E152" s="1" t="s">
         <v>608</v>
       </c>
-      <c r="F152" s="3">
+      <c r="F152" s="9">
         <v>45786</v>
       </c>
     </row>
@@ -6260,7 +6265,7 @@
       <c r="E153" s="1" t="s">
         <v>612</v>
       </c>
-      <c r="F153" s="3">
+      <c r="F153" s="9">
         <v>45788</v>
       </c>
     </row>
@@ -6281,7 +6286,7 @@
       <c r="E154" s="1" t="s">
         <v>616</v>
       </c>
-      <c r="F154" s="3">
+      <c r="F154" s="9">
         <v>45979</v>
       </c>
     </row>
@@ -6302,7 +6307,7 @@
       <c r="E155" s="1" t="s">
         <v>620</v>
       </c>
-      <c r="F155" s="3">
+      <c r="F155" s="9">
         <v>45799</v>
       </c>
     </row>
@@ -6323,7 +6328,7 @@
       <c r="E156" s="1" t="s">
         <v>624</v>
       </c>
-      <c r="F156" s="3">
+      <c r="F156" s="9">
         <v>45801</v>
       </c>
     </row>
@@ -6344,7 +6349,7 @@
       <c r="E157" s="1" t="s">
         <v>628</v>
       </c>
-      <c r="F157" s="3">
+      <c r="F157" s="9">
         <v>45803</v>
       </c>
     </row>
@@ -6365,7 +6370,7 @@
       <c r="E158" s="1" t="s">
         <v>632</v>
       </c>
-      <c r="F158" s="3">
+      <c r="F158" s="9">
         <v>45805</v>
       </c>
     </row>
@@ -6386,7 +6391,7 @@
       <c r="E159" s="1" t="s">
         <v>636</v>
       </c>
-      <c r="F159" s="3">
+      <c r="F159" s="9">
         <v>45807</v>
       </c>
     </row>
@@ -6407,7 +6412,7 @@
       <c r="E160" s="1" t="s">
         <v>640</v>
       </c>
-      <c r="F160" s="3">
+      <c r="F160" s="9">
         <v>45817</v>
       </c>
     </row>
@@ -6428,7 +6433,7 @@
       <c r="E161" s="1" t="s">
         <v>644</v>
       </c>
-      <c r="F161" s="3">
+      <c r="F161" s="9">
         <v>45821</v>
       </c>
     </row>
@@ -6449,7 +6454,7 @@
       <c r="E162" s="1" t="s">
         <v>648</v>
       </c>
-      <c r="F162" s="3">
+      <c r="F162" s="9">
         <v>45824</v>
       </c>
     </row>
@@ -6470,7 +6475,7 @@
       <c r="E163" s="1" t="s">
         <v>652</v>
       </c>
-      <c r="F163" s="3">
+      <c r="F163" s="9">
         <v>45827</v>
       </c>
     </row>
@@ -6491,7 +6496,7 @@
       <c r="E164" s="1" t="s">
         <v>656</v>
       </c>
-      <c r="F164" s="3">
+      <c r="F164" s="9">
         <v>45836</v>
       </c>
     </row>
@@ -6512,7 +6517,7 @@
       <c r="E165" s="1" t="s">
         <v>660</v>
       </c>
-      <c r="F165" s="3">
+      <c r="F165" s="9">
         <v>45844</v>
       </c>
     </row>
@@ -6533,7 +6538,7 @@
       <c r="E166" s="1" t="s">
         <v>664</v>
       </c>
-      <c r="F166" s="3">
+      <c r="F166" s="9">
         <v>45849</v>
       </c>
     </row>
@@ -6554,7 +6559,7 @@
       <c r="E167" s="1" t="s">
         <v>668</v>
       </c>
-      <c r="F167" s="3">
+      <c r="F167" s="9">
         <v>45856</v>
       </c>
     </row>
@@ -6575,7 +6580,7 @@
       <c r="E168" s="1" t="s">
         <v>672</v>
       </c>
-      <c r="F168" s="3">
+      <c r="F168" s="9">
         <v>45871</v>
       </c>
     </row>
@@ -6596,7 +6601,7 @@
       <c r="E169" s="1" t="s">
         <v>676</v>
       </c>
-      <c r="F169" s="3">
+      <c r="F169" s="9">
         <v>45878</v>
       </c>
     </row>
@@ -6617,7 +6622,7 @@
       <c r="E170" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="F170" s="3">
+      <c r="F170" s="9">
         <v>45886</v>
       </c>
     </row>
@@ -6638,7 +6643,7 @@
       <c r="E171" s="1" t="s">
         <v>684</v>
       </c>
-      <c r="F171" s="3">
+      <c r="F171" s="9">
         <v>45888</v>
       </c>
     </row>
@@ -6659,7 +6664,7 @@
       <c r="E172" s="1" t="s">
         <v>688</v>
       </c>
-      <c r="F172" s="3">
+      <c r="F172" s="9">
         <v>45893</v>
       </c>
     </row>
@@ -6680,7 +6685,7 @@
       <c r="E173" s="1" t="s">
         <v>692</v>
       </c>
-      <c r="F173" s="2" t="s">
+      <c r="F173" s="8" t="s">
         <v>693</v>
       </c>
     </row>
@@ -6701,7 +6706,7 @@
       <c r="E174" s="1" t="s">
         <v>697</v>
       </c>
-      <c r="F174" s="5">
+      <c r="F174" s="11">
         <v>45933</v>
       </c>
     </row>
@@ -6722,7 +6727,7 @@
       <c r="E175" s="1" t="s">
         <v>701</v>
       </c>
-      <c r="F175" s="5">
+      <c r="F175" s="11">
         <v>45938</v>
       </c>
     </row>
@@ -6743,7 +6748,7 @@
       <c r="E176" s="1" t="s">
         <v>705</v>
       </c>
-      <c r="F176" s="5">
+      <c r="F176" s="11">
         <v>45945</v>
       </c>
     </row>
@@ -6755,16 +6760,16 @@
       <c r="B177" t="s">
         <v>706</v>
       </c>
-      <c r="C177" s="6" t="s">
+      <c r="C177" s="3" t="s">
         <v>707</v>
       </c>
-      <c r="D177" s="6" t="s">
+      <c r="D177" s="3" t="s">
         <v>708</v>
       </c>
-      <c r="E177" s="6" t="s">
+      <c r="E177" s="3" t="s">
         <v>709</v>
       </c>
-      <c r="F177" s="5">
+      <c r="F177" s="11">
         <v>45967</v>
       </c>
     </row>
@@ -6776,16 +6781,16 @@
       <c r="B178" t="s">
         <v>710</v>
       </c>
-      <c r="C178" s="6" t="s">
+      <c r="C178" s="3" t="s">
         <v>711</v>
       </c>
-      <c r="D178" s="6" t="s">
+      <c r="D178" s="3" t="s">
         <v>712</v>
       </c>
-      <c r="E178" s="6" t="s">
+      <c r="E178" s="3" t="s">
         <v>713</v>
       </c>
-      <c r="F178" s="5">
+      <c r="F178" s="11">
         <v>45964</v>
       </c>
     </row>
@@ -6806,7 +6811,7 @@
       <c r="E179" s="1" t="s">
         <v>717</v>
       </c>
-      <c r="F179" s="5">
+      <c r="F179" s="11">
         <v>45974</v>
       </c>
     </row>
@@ -6827,7 +6832,7 @@
       <c r="E180" s="1" t="s">
         <v>721</v>
       </c>
-      <c r="F180" s="5">
+      <c r="F180" s="11">
         <v>45975</v>
       </c>
     </row>
@@ -6848,7 +6853,7 @@
       <c r="E181" s="1" t="s">
         <v>725</v>
       </c>
-      <c r="F181" s="5">
+      <c r="F181" s="11">
         <v>45984</v>
       </c>
     </row>
@@ -6869,7 +6874,7 @@
       <c r="E182" s="1" t="s">
         <v>729</v>
       </c>
-      <c r="F182" s="5">
+      <c r="F182" s="11">
         <v>45982</v>
       </c>
     </row>
@@ -6890,7 +6895,7 @@
       <c r="E183" s="1" t="s">
         <v>733</v>
       </c>
-      <c r="F183" s="5">
+      <c r="F183" s="11">
         <v>45986</v>
       </c>
     </row>
@@ -6911,7 +6916,7 @@
       <c r="E184" s="1" t="s">
         <v>737</v>
       </c>
-      <c r="F184" s="5">
+      <c r="F184" s="11">
         <v>45991</v>
       </c>
     </row>
@@ -6932,7 +6937,7 @@
       <c r="E185" s="1" t="s">
         <v>741</v>
       </c>
-      <c r="F185" s="5">
+      <c r="F185" s="11">
         <v>45994</v>
       </c>
     </row>
@@ -6953,7 +6958,7 @@
       <c r="E186" s="1" t="s">
         <v>745</v>
       </c>
-      <c r="F186" s="5">
+      <c r="F186" s="11">
         <v>45997</v>
       </c>
     </row>
@@ -6974,7 +6979,7 @@
       <c r="E187" s="1" t="s">
         <v>749</v>
       </c>
-      <c r="F187" s="5">
+      <c r="F187" s="11">
         <v>46029</v>
       </c>
     </row>
@@ -6995,7 +7000,7 @@
       <c r="E188" s="1" t="s">
         <v>753</v>
       </c>
-      <c r="F188" s="5">
+      <c r="F188" s="11">
         <v>46039</v>
       </c>
     </row>
@@ -7016,7 +7021,7 @@
       <c r="E189" s="1" t="s">
         <v>757</v>
       </c>
-      <c r="F189" s="5">
+      <c r="F189" s="11">
         <v>46045</v>
       </c>
     </row>
@@ -7037,7 +7042,7 @@
       <c r="E190" s="1" t="s">
         <v>761</v>
       </c>
-      <c r="F190" s="5">
+      <c r="F190" s="11">
         <v>46049</v>
       </c>
     </row>
@@ -7058,7 +7063,7 @@
       <c r="E191" s="1" t="s">
         <v>765</v>
       </c>
-      <c r="F191" s="5">
+      <c r="F191" s="11">
         <v>46053</v>
       </c>
     </row>
@@ -7079,7 +7084,7 @@
       <c r="E192" s="1" t="s">
         <v>769</v>
       </c>
-      <c r="F192" s="5">
+      <c r="F192" s="11">
         <v>46057</v>
       </c>
     </row>
@@ -7100,7 +7105,7 @@
       <c r="E193" s="1" t="s">
         <v>773</v>
       </c>
-      <c r="F193" s="5">
+      <c r="F193" s="11">
         <v>46063</v>
       </c>
     </row>
@@ -7121,7 +7126,7 @@
       <c r="E194" s="1" t="s">
         <v>777</v>
       </c>
-      <c r="F194" s="5">
+      <c r="F194" s="11">
         <v>46072</v>
       </c>
     </row>
@@ -7142,7 +7147,7 @@
       <c r="E195" s="1" t="s">
         <v>781</v>
       </c>
-      <c r="F195" s="5">
+      <c r="F195" s="11">
         <v>46075</v>
       </c>
       <c r="G195" s="1"/>
@@ -7164,7 +7169,7 @@
       <c r="E196" s="1" t="s">
         <v>785</v>
       </c>
-      <c r="F196" s="5">
+      <c r="F196" s="11">
         <v>46081</v>
       </c>
     </row>
@@ -7185,7 +7190,7 @@
       <c r="E197" s="1" t="s">
         <v>789</v>
       </c>
-      <c r="F197" s="5">
+      <c r="F197" s="11">
         <v>46083</v>
       </c>
     </row>
@@ -7206,7 +7211,7 @@
       <c r="E198" s="1" t="s">
         <v>793</v>
       </c>
-      <c r="F198" s="5">
+      <c r="F198" s="11">
         <v>46087</v>
       </c>
     </row>
@@ -7223,10 +7228,10 @@
       <c r="D199" s="1" t="s">
         <v>796</v>
       </c>
-      <c r="E199" s="8" t="s">
+      <c r="E199" s="5" t="s">
         <v>797</v>
       </c>
-      <c r="F199" s="5">
+      <c r="F199" s="11">
         <v>46092</v>
       </c>
     </row>
@@ -7243,10 +7248,10 @@
       <c r="D200" s="1" t="s">
         <v>800</v>
       </c>
-      <c r="E200" s="8" t="s">
+      <c r="E200" s="5" t="s">
         <v>801</v>
       </c>
-      <c r="F200" s="8">
+      <c r="F200" s="11">
         <v>46095</v>
       </c>
     </row>
@@ -7266,7 +7271,7 @@
       <c r="E201" t="s">
         <v>802</v>
       </c>
-      <c r="F201" s="5">
+      <c r="F201" s="11">
         <v>46098</v>
       </c>
     </row>
@@ -7303,7 +7308,7 @@
       <c r="E203" t="s">
         <v>811</v>
       </c>
-      <c r="F203" s="5">
+      <c r="F203" s="11">
         <v>46103</v>
       </c>
     </row>
@@ -7320,10 +7325,10 @@
       <c r="D204" s="1" t="s">
         <v>813</v>
       </c>
-      <c r="E204" s="9" t="s">
+      <c r="E204" s="6" t="s">
         <v>814</v>
       </c>
-      <c r="F204" s="8">
+      <c r="F204" s="11">
         <v>46106</v>
       </c>
     </row>
@@ -7343,7 +7348,7 @@
       <c r="E205" t="s">
         <v>819</v>
       </c>
-      <c r="F205" s="10">
+      <c r="F205" s="12">
         <v>46111</v>
       </c>
     </row>
@@ -7363,7 +7368,7 @@
       <c r="E206" t="s">
         <v>820</v>
       </c>
-      <c r="F206" s="5">
+      <c r="F206" s="11">
         <v>46112</v>
       </c>
     </row>
@@ -7383,7 +7388,7 @@
       <c r="E207" t="s">
         <v>830</v>
       </c>
-      <c r="F207" s="5">
+      <c r="F207" s="11">
         <v>46118</v>
       </c>
     </row>
@@ -7403,7 +7408,7 @@
       <c r="E208" t="s">
         <v>831</v>
       </c>
-      <c r="F208" s="5">
+      <c r="F208" s="11">
         <v>46121</v>
       </c>
     </row>
@@ -7423,7 +7428,7 @@
       <c r="E209" t="s">
         <v>832</v>
       </c>
-      <c r="F209" s="5">
+      <c r="F209" s="11">
         <v>46122</v>
       </c>
     </row>
@@ -7443,7 +7448,7 @@
       <c r="E210" t="s">
         <v>843</v>
       </c>
-      <c r="F210" s="10">
+      <c r="F210" s="12">
         <v>46126</v>
       </c>
     </row>
@@ -7463,7 +7468,7 @@
       <c r="E211" t="s">
         <v>842</v>
       </c>
-      <c r="F211" s="10">
+      <c r="F211" s="12">
         <v>46128</v>
       </c>
     </row>
@@ -7483,7 +7488,7 @@
       <c r="E212" t="s">
         <v>847</v>
       </c>
-      <c r="F212" s="5">
+      <c r="F212" s="11">
         <v>45463</v>
       </c>
     </row>
@@ -7503,7 +7508,7 @@
       <c r="E213" t="s">
         <v>851</v>
       </c>
-      <c r="F213" s="5">
+      <c r="F213" s="11">
         <v>46137</v>
       </c>
     </row>
@@ -7520,10 +7525,10 @@
       <c r="D214" s="1" t="s">
         <v>854</v>
       </c>
-      <c r="E214" s="11" t="s">
+      <c r="E214" s="7" t="s">
         <v>855</v>
       </c>
-      <c r="F214" s="10">
+      <c r="F214" s="12">
         <v>46140</v>
       </c>
     </row>
@@ -7543,11 +7548,14 @@
       <c r="E215" t="s">
         <v>859</v>
       </c>
-      <c r="F215" s="5">
+      <c r="F215" s="11">
         <v>46163</v>
       </c>
     </row>
     <row r="216" spans="1:6" ht="213.75" x14ac:dyDescent="0.2">
+      <c r="A216">
+        <v>215</v>
+      </c>
       <c r="B216" t="s">
         <v>860</v>
       </c>
@@ -7560,8 +7568,28 @@
       <c r="E216" t="s">
         <v>863</v>
       </c>
-      <c r="F216" s="5">
+      <c r="F216" s="11">
         <v>46165</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6" ht="242.25" x14ac:dyDescent="0.2">
+      <c r="A217">
+        <v>216</v>
+      </c>
+      <c r="B217" t="s">
+        <v>864</v>
+      </c>
+      <c r="C217" s="1" t="s">
+        <v>865</v>
+      </c>
+      <c r="D217" s="1" t="s">
+        <v>866</v>
+      </c>
+      <c r="E217" s="5" t="s">
+        <v>867</v>
+      </c>
+      <c r="F217" s="11">
+        <v>46172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add inner report image data
</commit_message>
<xml_diff>
--- a/data/image_data.xlsx
+++ b/data/image_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Programming\MyCellphoeApp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C7B3994-EAC9-4FBA-B30B-6F57D9536E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{283CFB9C-8D6B-4580-ACBB-0A2A8FC9885C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="877">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="881">
   <si>
     <t>Number</t>
   </si>
@@ -2651,6 +2651,18 @@
   </si>
   <si>
     <t xml:space="preserve">What happens when you discover that your own life has already been written? </t>
+  </si>
+  <si>
+    <t>The Inner Report</t>
+  </si>
+  <si>
+    <t>The image presents a dark, cinematic interior divided between two visual worlds: on the left, a television broadcasts a cheerful “Breaking News” report about a hot air balloon festival, complete with bright colors, celebratory scenery, and the familiar visual language of televised optimism. On the right, a giant anatomical cross-section of a human eye dominates the room, its interior transformed into a burning landscape of war, ruins, explosions, and destruction. Inside the eye itself, a small elderly man sits quietly in an armchair, facing the television from within the devastated inner chamber. The contrast is striking: the external screen reports harmless festivity, while the inner eye contains catastrophe. The polished floor reflects both the cold blue light of the television and the fiery orange glow of destruction, binding the two realities into one psychological space.</t>
+  </si>
+  <si>
+    <t>The image strongly suggests a split between public narrative and private perception. The television represents the outer report: packaged, simplified, cheerful, and consumable. The eye, however, contains the inner report: the unfiltered psychic reality of anxiety, memory, trauma, or dread. The seated figure inside the eye becomes an internal witness, someone unable to escape what he sees or remembers, even while the world outside continues to broadcast distraction and celebration. The hot air balloon festival is especially effective because it implies lightness, elevation, and innocence, while the retinal landscape shows gravity, collapse, and burning. The work therefore becomes a meditation on perception itself: what we are told to see versus what we actually carry inside. It also suggests that the eye is not merely an organ of vision, but a chamber of interpretation, where every external image is transformed by accumulated fear, history, and personal vulnerability.</t>
+  </si>
+  <si>
+    <t>What private catastrophe do you see while the world reports only celebration?</t>
   </si>
 </sst>
 </file>
@@ -3014,7 +3026,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G219"/>
+  <dimension ref="A1:G220"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -7393,6 +7405,26 @@
         <v>46181</v>
       </c>
     </row>
+    <row r="220" spans="1:6" ht="185.25" x14ac:dyDescent="0.2">
+      <c r="A220">
+        <v>219</v>
+      </c>
+      <c r="B220" t="s">
+        <v>877</v>
+      </c>
+      <c r="C220" s="1" t="s">
+        <v>878</v>
+      </c>
+      <c r="D220" s="1" t="s">
+        <v>879</v>
+      </c>
+      <c r="E220" t="s">
+        <v>880</v>
+      </c>
+      <c r="F220" s="4">
+        <v>46185</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Add missing gallery images
</commit_message>
<xml_diff>
--- a/data/image_data.xlsx
+++ b/data/image_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Programming\MyCellphoeApp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8DB204-9194-417A-A80C-9A43507AA5D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{863DD3BD-28A5-448E-A60C-4D7782835FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="910">
   <si>
     <t>Number</t>
   </si>
@@ -2726,6 +2726,30 @@
   </si>
   <si>
     <t>What part of your life is still falling, even though it ended long ago?</t>
+  </si>
+  <si>
+    <t>Breakfast Over The Bahai Temple</t>
+  </si>
+  <si>
+    <t>A solitary man enjoys a simple breakfast at a modest white table suspended impossibly above a panoramic view of Haifa and the Baháʼí Gardens, while the Earth curves gently beneath a star-filled sky. Around him float the planets of the Solar System, transforming the familiar morning ritual into a cosmic event. A single hanging light bulb illuminates the table, where coffee, cheese, vegetables, and bread suggest the quiet intimacy of an ordinary meal. Barely acknowledging the spectacular universe surrounding him, the man remains focused on his breakfast, creating a striking contrast between the immensity of the cosmos and the simplicity of everyday life.</t>
+  </si>
+  <si>
+    <t>This image examines the relationship between the ordinary and the infinite, suggesting that human existence unfolds simultaneously on two vastly different scales. While the surrounding planets and the Milky Way evoke the incomprehensible magnitude of the universe, the figure remains absorbed in one of life's most routine activities. Rather than diminishing the breakfast, the cosmic setting elevates it, proposing that meaning is not found only in extraordinary discoveries but also in the quiet rituals that structure our lives. The image challenges the viewer to consider whether the universe derives significance from its immense scale or whether significance is instead created through conscious human experience. By placing an everyday meal above a recognizable earthly landscape and beneath an infinite sky, the work celebrates the coexistence of wonder and routine, reminding us that even the most mundane moments occur within a universe of staggering beauty and mystery.</t>
+  </si>
+  <si>
+    <t>Can you remain present in ordinary moments while surrounded by life's overwhelming vastness?</t>
+  </si>
+  <si>
+    <t>A Visit To My Unlived Youth Fantasies Gallery</t>
+  </si>
+  <si>
+    <t>The image presents a dimly lit, museum-like gallery with dark green walls, reflective floors, ornate gold frames, and a strong perspective that draws the eye into the distance. In the foreground, an older, bald man wearing a black tuxedo and holding a champagne glass turns toward the viewer while surveying a long sequence of imagined scenes. The framed images portray extraordinary versions of life—basketball triumph, romantic glamour, motor racing, flight, space exploration, mountain adventure, and other feats of daring and achievement. Carefully positioned spotlights illuminate each picture, giving the fantasies the status of prized cultural artifacts or preserved memories.</t>
+  </si>
+  <si>
+    <t>The work explores the relationship between aging, memory, desire, and the alternative lives a person imagines but never experiences. The gallery functions as an inner psychological space: each framed image represents a possible identity, while the older man appears both as spectator and curator of his own unrealized history. His tuxedo and champagne suggest sophistication, success, and social recognition, yet his solitary position and slightly distant expression introduce a sense of reflection, absence, or regret. The contrast between his stillness and the dynamic scenes behind him emphasizes the gap between the life he is living and the youthful fantasies that remain emotionally vivid. The image therefore asks whether imagination can preserve lost possibilities, or whether it ultimately reminds us of the selves we were unable—or unwilling—to become.</t>
+  </si>
+  <si>
+    <t>An aging man studies unrealized adventures: which forgotten self still seeks recognition?</t>
   </si>
 </sst>
 </file>
@@ -3092,7 +3116,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L225"/>
+  <dimension ref="A1:L227"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -7600,6 +7624,46 @@
         <v>46214</v>
       </c>
     </row>
+    <row r="226" spans="1:6" ht="185.25" x14ac:dyDescent="0.2">
+      <c r="A226">
+        <v>225</v>
+      </c>
+      <c r="B226" t="s">
+        <v>902</v>
+      </c>
+      <c r="C226" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="D226" s="1" t="s">
+        <v>904</v>
+      </c>
+      <c r="E226" t="s">
+        <v>905</v>
+      </c>
+      <c r="F226" s="4">
+        <v>46216</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" ht="156.75" x14ac:dyDescent="0.2">
+      <c r="A227">
+        <v>226</v>
+      </c>
+      <c r="B227" t="s">
+        <v>906</v>
+      </c>
+      <c r="C227" s="1" t="s">
+        <v>907</v>
+      </c>
+      <c r="D227" s="1" t="s">
+        <v>908</v>
+      </c>
+      <c r="E227" t="s">
+        <v>909</v>
+      </c>
+      <c r="F227" s="4">
+        <v>46221</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Add missing gallery images (#1)
Regenerate image data and add the two missing JPEG files.
</commit_message>
<xml_diff>
--- a/data/image_data.xlsx
+++ b/data/image_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Programming\MyCellphoeApp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8DB204-9194-417A-A80C-9A43507AA5D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{863DD3BD-28A5-448E-A60C-4D7782835FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="910">
   <si>
     <t>Number</t>
   </si>
@@ -2726,6 +2726,30 @@
   </si>
   <si>
     <t>What part of your life is still falling, even though it ended long ago?</t>
+  </si>
+  <si>
+    <t>Breakfast Over The Bahai Temple</t>
+  </si>
+  <si>
+    <t>A solitary man enjoys a simple breakfast at a modest white table suspended impossibly above a panoramic view of Haifa and the Baháʼí Gardens, while the Earth curves gently beneath a star-filled sky. Around him float the planets of the Solar System, transforming the familiar morning ritual into a cosmic event. A single hanging light bulb illuminates the table, where coffee, cheese, vegetables, and bread suggest the quiet intimacy of an ordinary meal. Barely acknowledging the spectacular universe surrounding him, the man remains focused on his breakfast, creating a striking contrast between the immensity of the cosmos and the simplicity of everyday life.</t>
+  </si>
+  <si>
+    <t>This image examines the relationship between the ordinary and the infinite, suggesting that human existence unfolds simultaneously on two vastly different scales. While the surrounding planets and the Milky Way evoke the incomprehensible magnitude of the universe, the figure remains absorbed in one of life's most routine activities. Rather than diminishing the breakfast, the cosmic setting elevates it, proposing that meaning is not found only in extraordinary discoveries but also in the quiet rituals that structure our lives. The image challenges the viewer to consider whether the universe derives significance from its immense scale or whether significance is instead created through conscious human experience. By placing an everyday meal above a recognizable earthly landscape and beneath an infinite sky, the work celebrates the coexistence of wonder and routine, reminding us that even the most mundane moments occur within a universe of staggering beauty and mystery.</t>
+  </si>
+  <si>
+    <t>Can you remain present in ordinary moments while surrounded by life's overwhelming vastness?</t>
+  </si>
+  <si>
+    <t>A Visit To My Unlived Youth Fantasies Gallery</t>
+  </si>
+  <si>
+    <t>The image presents a dimly lit, museum-like gallery with dark green walls, reflective floors, ornate gold frames, and a strong perspective that draws the eye into the distance. In the foreground, an older, bald man wearing a black tuxedo and holding a champagne glass turns toward the viewer while surveying a long sequence of imagined scenes. The framed images portray extraordinary versions of life—basketball triumph, romantic glamour, motor racing, flight, space exploration, mountain adventure, and other feats of daring and achievement. Carefully positioned spotlights illuminate each picture, giving the fantasies the status of prized cultural artifacts or preserved memories.</t>
+  </si>
+  <si>
+    <t>The work explores the relationship between aging, memory, desire, and the alternative lives a person imagines but never experiences. The gallery functions as an inner psychological space: each framed image represents a possible identity, while the older man appears both as spectator and curator of his own unrealized history. His tuxedo and champagne suggest sophistication, success, and social recognition, yet his solitary position and slightly distant expression introduce a sense of reflection, absence, or regret. The contrast between his stillness and the dynamic scenes behind him emphasizes the gap between the life he is living and the youthful fantasies that remain emotionally vivid. The image therefore asks whether imagination can preserve lost possibilities, or whether it ultimately reminds us of the selves we were unable—or unwilling—to become.</t>
+  </si>
+  <si>
+    <t>An aging man studies unrealized adventures: which forgotten self still seeks recognition?</t>
   </si>
 </sst>
 </file>
@@ -3092,7 +3116,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L225"/>
+  <dimension ref="A1:L227"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -7600,6 +7624,46 @@
         <v>46214</v>
       </c>
     </row>
+    <row r="226" spans="1:6" ht="185.25" x14ac:dyDescent="0.2">
+      <c r="A226">
+        <v>225</v>
+      </c>
+      <c r="B226" t="s">
+        <v>902</v>
+      </c>
+      <c r="C226" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="D226" s="1" t="s">
+        <v>904</v>
+      </c>
+      <c r="E226" t="s">
+        <v>905</v>
+      </c>
+      <c r="F226" s="4">
+        <v>46216</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" ht="156.75" x14ac:dyDescent="0.2">
+      <c r="A227">
+        <v>226</v>
+      </c>
+      <c r="B227" t="s">
+        <v>906</v>
+      </c>
+      <c r="C227" s="1" t="s">
+        <v>907</v>
+      </c>
+      <c r="D227" s="1" t="s">
+        <v>908</v>
+      </c>
+      <c r="E227" t="s">
+        <v>909</v>
+      </c>
+      <c r="F227" s="4">
+        <v>46221</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>